<commit_message>
Stage 8 review fixes: D-008
</commit_message>
<xml_diff>
--- a/output/archive/QuenverellData/engagements/dt-6/docking/tautomers/dt6-docking-hitlist-2013-11-06.xlsx
+++ b/output/archive/QuenverellData/engagements/dt-6/docking/tautomers/dt6-docking-hitlist-2013-11-06.xlsx
@@ -154,7 +154,7 @@
   <commentList>
     <comment ref="B3" authorId="0" shapeId="0">
       <text>
-        <t>Check the second protonation set against the preparation log before we rerun the clusters</t>
+        <t>Use the reviewed preparation record alongside the docking run records.</t>
       </text>
     </comment>
   </commentList>
@@ -611,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -625,113 +625,86 @@
           <t>Step</t>
         </is>
       </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Source record</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Interpretation</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ligand preparation</t>
+          <t>Preparation</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Protonation states generated at pH 7.4, with a second set at pH 6.0 for ligands carrying an ionisable amine</t>
+          <t>Preparation and protonation-state records in the engagement file</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Second set added after the protonation-state review; see Consensus</t>
+          <t>Use reviewed states to interpret hit order</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Conformers</t>
+          <t>Docking</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Up to 10 per ligand, RMSD cut-off 0.5 Å</t>
+          <t>Run settings and provenance in the engagement records</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Conformer set kept with the run files</t>
+          <t>Scores in kcal/mol support triage, not measured affinity</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Receptor grid</t>
+          <t>Protonation review</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Box centred on the binding site defined in the client's receptor model, 22 Å edge</t>
+          <t>Review accompanying the DT-6 readout</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Receptor model supplied by Drelvessa; Quenverell did not alter it</t>
+          <t>The review changed the hit ranking</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Docking</t>
+          <t>Hit clustering</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Best pose per ligand retained for each protonation set</t>
+          <t>Clustering record accompanying the readout</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Scores in kcal/mol</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Clustering</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Hit clustering on fingerprint similarity, Butina cut-off</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Clusters used to pick diverse hits for the candidate set</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Reference run</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Known binders docked with the same settings before the library run</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Used to confirm the grid reproduces the expected pose</t>
+          <t>Consider alongside the ranking</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -771,7 +744,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Consensus of the two protonation sets, ranked on the better of the two best scores per ligand</t>
+          <t>Consensus ranking following the protonation-state review; method and compound identities are retained in the engagement records.</t>
         </is>
       </c>
     </row>

</xml_diff>